<commit_message>
Run all 288 HR beam cases (S355/S460/S690) and drop material .dat files
- 1.-4. .dat inputs extended to 288 rows (Fy = 355, 460, 690 MPa)
- noCUFSM generator: loop over all rows, cpus=20, delete .odb after
  extraction, write section properties to parameters_section_All.xlsx
  (no longer overwrites parameters_section_HEB.xlsx)
- remove 5./6./7. material .dat files (law now generated in the code)
- remove old validation spreadsheets/figures and test_calibration figures
- add aluminum 3PB test output, material_behavior.pdf (Yun & Gardner 2017)
- update input/result workbooks

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrainte_residuelle.xlsx
+++ b/Contrainte_residuelle.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Kokou\Kokou_Case_study_1_Steel_Column\Numerical model_validation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1447F4F-BC96-476B-8EB9-E0D618B693A0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B825A4C4-81A6-4A0F-B8B7-1C9F5778890B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029" iterate="1" concurrentCalc="0"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -453,17 +452,17 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C2FB0444-6390-4291-91EC-7047928FBF0F}">
   <dimension ref="A1:BC97"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="3.140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="12.28515625" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="11.5703125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="3.1796875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="4" width="11.54296875" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="12" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
-    <col min="13" max="13" width="12.7109375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="12.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -483,7 +482,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -506,146 +505,32 @@
         <f>F2*G2</f>
         <v>1351.0206340923255</v>
       </c>
-      <c r="J2">
-        <v>24.884398168940699</v>
-      </c>
-      <c r="K2">
-        <v>53.8206018310593</v>
-      </c>
-      <c r="L2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="M2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="N2">
-        <v>81.377999999999801</v>
-      </c>
-      <c r="O2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="P2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="Q2">
-        <v>81.377999999999801</v>
-      </c>
-      <c r="R2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="S2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="T2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="U2">
-        <v>81.377999999999901</v>
-      </c>
-      <c r="V2">
-        <v>53.820601831059399</v>
-      </c>
-      <c r="W2">
-        <v>24.884398168940599</v>
-      </c>
-      <c r="X2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="Y2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="Z2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AA2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AB2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AC2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AD2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AE2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AF2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AG2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AH2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AI2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AJ2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AK2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AL2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AM2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AN2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AO2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AP2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AQ2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AR2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AS2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AT2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AU2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AV2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AW2">
-        <v>64.552499999999895</v>
-      </c>
-      <c r="AX2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AY2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="AZ2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="BA2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="BB2" s="1">
-        <v>120.9825</v>
-      </c>
-      <c r="BC2" s="1">
-        <v>120.9825</v>
-      </c>
-    </row>
-    <row r="3" spans="1:55" x14ac:dyDescent="0.25">
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
+      <c r="AB2" s="1"/>
+      <c r="AC2" s="1"/>
+      <c r="AH2" s="1"/>
+      <c r="AI2" s="1"/>
+      <c r="AJ2" s="1"/>
+      <c r="AK2" s="1"/>
+      <c r="AL2" s="1"/>
+      <c r="AM2" s="1"/>
+      <c r="AN2" s="1"/>
+      <c r="AO2" s="1"/>
+      <c r="AP2" s="1"/>
+      <c r="AQ2" s="1"/>
+      <c r="AR2" s="1"/>
+      <c r="AS2" s="1"/>
+      <c r="AX2" s="1"/>
+      <c r="AY2" s="1"/>
+      <c r="AZ2" s="1"/>
+      <c r="BA2" s="1"/>
+      <c r="BB2" s="1"/>
+      <c r="BC2" s="1"/>
+    </row>
+    <row r="3" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>2</v>
       </c>
@@ -669,7 +554,7 @@
         <v>2204.133829473014</v>
       </c>
     </row>
-    <row r="4" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>3</v>
       </c>
@@ -693,7 +578,7 @@
         <v>1687.9866410823936</v>
       </c>
     </row>
-    <row r="5" spans="1:55" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>4</v>
       </c>
@@ -716,14 +601,8 @@
         <f t="shared" si="0"/>
         <v>76.741054481946222</v>
       </c>
-      <c r="M5">
-        <v>1351.0206340923255</v>
-      </c>
-      <c r="N5">
-        <v>24.884398168940699</v>
-      </c>
-    </row>
-    <row r="6" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>5</v>
       </c>
@@ -746,14 +625,8 @@
         <f t="shared" si="0"/>
         <v>-1131.6931354683907</v>
       </c>
-      <c r="M6">
-        <v>2204.133829473014</v>
-      </c>
-      <c r="N6">
-        <v>53.8206018310593</v>
-      </c>
-    </row>
-    <row r="7" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>6</v>
       </c>
@@ -776,14 +649,8 @@
         <f t="shared" si="0"/>
         <v>-1937.3159287686176</v>
       </c>
-      <c r="M7">
-        <v>1687.9866410823936</v>
-      </c>
-      <c r="N7">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="8" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>7</v>
       </c>
@@ -806,14 +673,8 @@
         <f t="shared" si="0"/>
         <v>-2340.1273254187263</v>
       </c>
-      <c r="M8">
-        <v>76.741054481946222</v>
-      </c>
-      <c r="N8">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="9" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>8</v>
       </c>
@@ -836,14 +697,8 @@
         <f t="shared" si="0"/>
         <v>-2340.1273254187236</v>
       </c>
-      <c r="M9">
-        <v>-1131.6931354683907</v>
-      </c>
-      <c r="N9">
-        <v>81.377999999999801</v>
-      </c>
-    </row>
-    <row r="10" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>9</v>
       </c>
@@ -866,14 +721,8 @@
         <f t="shared" si="0"/>
         <v>-1937.3159287686176</v>
       </c>
-      <c r="M10">
-        <v>-1937.3159287686176</v>
-      </c>
-      <c r="N10">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="11" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>10</v>
       </c>
@@ -896,14 +745,8 @@
         <f t="shared" si="0"/>
         <v>-1131.693135468392</v>
       </c>
-      <c r="M11">
-        <v>-2340.1273254187263</v>
-      </c>
-      <c r="N11">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="12" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>11</v>
       </c>
@@ -926,14 +769,8 @@
         <f t="shared" si="0"/>
         <v>76.741054481946222</v>
       </c>
-      <c r="M12">
-        <v>-2340.1273254187236</v>
-      </c>
-      <c r="N12">
-        <v>81.377999999999801</v>
-      </c>
-    </row>
-    <row r="13" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>12</v>
       </c>
@@ -956,14 +793,8 @@
         <f t="shared" si="0"/>
         <v>1687.9866410823936</v>
       </c>
-      <c r="M13">
-        <v>-1937.3159287686176</v>
-      </c>
-      <c r="N13">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="14" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>13</v>
       </c>
@@ -986,14 +817,8 @@
         <f t="shared" si="0"/>
         <v>2204.1338294730181</v>
       </c>
-      <c r="M14">
-        <v>-1131.693135468392</v>
-      </c>
-      <c r="N14">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="15" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>14</v>
       </c>
@@ -1016,14 +841,8 @@
         <f t="shared" si="0"/>
         <v>1351.0206340923203</v>
       </c>
-      <c r="M15">
-        <v>76.741054481946222</v>
-      </c>
-      <c r="N15">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="16" spans="1:55" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:55" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>15</v>
       </c>
@@ -1046,14 +865,8 @@
         <f t="shared" si="0"/>
         <v>-11304.950252296278</v>
       </c>
-      <c r="M16">
-        <v>1687.9866410823936</v>
-      </c>
-      <c r="N16">
-        <v>81.377999999999901</v>
-      </c>
-    </row>
-    <row r="17" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>16</v>
       </c>
@@ -1076,14 +889,8 @@
         <f t="shared" si="0"/>
         <v>-6124.3698862916017</v>
       </c>
-      <c r="M17">
-        <v>2204.1338294730181</v>
-      </c>
-      <c r="N17">
-        <v>53.820601831059399</v>
-      </c>
-    </row>
-    <row r="18" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>17</v>
       </c>
@@ -1106,14 +913,8 @@
         <f t="shared" si="0"/>
         <v>-1797.6650261572265</v>
       </c>
-      <c r="M18">
-        <v>1351.0206340923203</v>
-      </c>
-      <c r="N18">
-        <v>24.884398168940599</v>
-      </c>
-    </row>
-    <row r="19" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>18</v>
       </c>
@@ -1136,16 +937,8 @@
         <f t="shared" si="0"/>
         <v>1675.1643281068239</v>
       </c>
-      <c r="M19">
-        <f>SUM(M5:M18)</f>
-        <v>-178.50846105211053</v>
-      </c>
-      <c r="N19">
-        <f>SUM(N5:N18)</f>
-        <v>971.18999999999903</v>
-      </c>
-    </row>
-    <row r="20" spans="1:14" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>19</v>
       </c>
@@ -1169,7 +962,7 @@
         <v>4294.118176500574</v>
       </c>
     </row>
-    <row r="21" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>20</v>
       </c>
@@ -1193,7 +986,7 @@
         <v>6059.1965190240116</v>
       </c>
     </row>
-    <row r="22" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>21</v>
       </c>
@@ -1217,7 +1010,7 @@
         <v>3646.5381007716737</v>
       </c>
     </row>
-    <row r="23" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>22</v>
       </c>
@@ -1241,7 +1034,7 @@
         <v>3776.2459000857361</v>
       </c>
     </row>
-    <row r="24" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>23</v>
       </c>
@@ -1265,7 +1058,7 @@
         <v>3776.2459000857361</v>
       </c>
     </row>
-    <row r="25" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>24</v>
       </c>
@@ -1289,7 +1082,7 @@
         <v>3646.5381007716737</v>
       </c>
     </row>
-    <row r="26" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>25</v>
       </c>
@@ -1313,7 +1106,7 @@
         <v>6059.1965190240235</v>
       </c>
     </row>
-    <row r="27" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -1337,7 +1130,7 @@
         <v>4294.1181765005858</v>
       </c>
     </row>
-    <row r="28" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>27</v>
       </c>
@@ -1361,7 +1154,7 @@
         <v>1675.1643281068359</v>
       </c>
     </row>
-    <row r="29" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>28</v>
       </c>
@@ -1385,7 +1178,7 @@
         <v>-1797.6650261572265</v>
       </c>
     </row>
-    <row r="30" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>29</v>
       </c>
@@ -1409,7 +1202,7 @@
         <v>-6124.3698862916017</v>
       </c>
     </row>
-    <row r="31" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>30</v>
       </c>
@@ -1433,7 +1226,7 @@
         <v>-11304.950252296278</v>
       </c>
     </row>
-    <row r="32" spans="1:14" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>31</v>
       </c>
@@ -1457,7 +1250,7 @@
         <v>-11304.950252296278</v>
       </c>
     </row>
-    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>32</v>
       </c>
@@ -1481,7 +1274,7 @@
         <v>-6124.3698862916017</v>
       </c>
     </row>
-    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>33</v>
       </c>
@@ -1505,7 +1298,7 @@
         <v>-1797.6650261572265</v>
       </c>
     </row>
-    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>34</v>
       </c>
@@ -1529,7 +1322,7 @@
         <v>1675.1643281068239</v>
       </c>
     </row>
-    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>35</v>
       </c>
@@ -1553,7 +1346,7 @@
         <v>4294.118176500574</v>
       </c>
     </row>
-    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>36</v>
       </c>
@@ -1577,7 +1370,7 @@
         <v>6059.1965190240116</v>
       </c>
     </row>
-    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>37</v>
       </c>
@@ -1601,7 +1394,7 @@
         <v>3646.5381007716737</v>
       </c>
     </row>
-    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>38</v>
       </c>
@@ -1625,7 +1418,7 @@
         <v>3776.2459000857361</v>
       </c>
     </row>
-    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>39</v>
       </c>
@@ -1649,7 +1442,7 @@
         <v>3776.2459000857361</v>
       </c>
     </row>
-    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>40</v>
       </c>
@@ -1673,7 +1466,7 @@
         <v>3646.5381007716737</v>
       </c>
     </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>41</v>
       </c>
@@ -1697,7 +1490,7 @@
         <v>6059.1965190240235</v>
       </c>
     </row>
-    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>42</v>
       </c>
@@ -1721,7 +1514,7 @@
         <v>4294.1181765005858</v>
       </c>
     </row>
-    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>43</v>
       </c>
@@ -1745,7 +1538,7 @@
         <v>1675.1643281068359</v>
       </c>
     </row>
-    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>44</v>
       </c>
@@ -1769,7 +1562,7 @@
         <v>-1797.6650261572265</v>
       </c>
     </row>
-    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>45</v>
       </c>
@@ -1793,7 +1586,7 @@
         <v>-6124.3698862916017</v>
       </c>
     </row>
-    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>46</v>
       </c>
@@ -1817,7 +1610,7 @@
         <v>-11304.950252296278</v>
       </c>
     </row>
-    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>47</v>
       </c>
@@ -1831,7 +1624,7 @@
         <v>1943.9953103585158</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>48</v>
       </c>
@@ -1845,7 +1638,7 @@
         <v>1943.9953103585158</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>49</v>
       </c>
@@ -1859,7 +1652,7 @@
         <v>1492.5597014307132</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>50</v>
       </c>
@@ -1873,7 +1666,7 @@
         <v>1492.5597014307132</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>51</v>
       </c>
@@ -1887,7 +1680,7 @@
         <v>2951.2138027013334</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>52</v>
       </c>
@@ -1901,7 +1694,7 @@
         <v>2951.2138027013334</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>53</v>
       </c>
@@ -1915,7 +1708,7 @@
         <v>2951.2138027013334</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>54</v>
       </c>
@@ -1929,7 +1722,7 @@
         <v>2951.2138027013334</v>
       </c>
     </row>
-    <row r="56" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>55</v>
       </c>
@@ -1943,7 +1736,7 @@
         <v>2951.2138027013334</v>
       </c>
     </row>
-    <row r="57" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>56</v>
       </c>
@@ -1957,7 +1750,7 @@
         <v>2951.2138027013334</v>
       </c>
     </row>
-    <row r="58" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>57</v>
       </c>
@@ -1971,7 +1764,7 @@
         <v>1294.2762975520636</v>
       </c>
     </row>
-    <row r="59" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>58</v>
       </c>
@@ -1985,7 +1778,7 @@
         <v>1294.2762975520636</v>
       </c>
     </row>
-    <row r="60" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>59</v>
       </c>
@@ -1999,7 +1792,7 @@
         <v>2106.9585174889135</v>
       </c>
     </row>
-    <row r="61" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>60</v>
       </c>
@@ -2013,7 +1806,7 @@
         <v>2106.9585174889135</v>
       </c>
     </row>
-    <row r="62" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>61</v>
       </c>
@@ -2027,7 +1820,7 @@
         <v>2106.9585174889135</v>
       </c>
     </row>
-    <row r="63" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>62</v>
       </c>
@@ -2041,7 +1834,7 @@
         <v>2106.9585174889135</v>
       </c>
     </row>
-    <row r="64" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>63</v>
       </c>
@@ -2055,7 +1848,7 @@
         <v>2106.9585174889135</v>
       </c>
     </row>
-    <row r="65" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>64</v>
       </c>
@@ -2069,7 +1862,7 @@
         <v>2106.9585174889135</v>
       </c>
     </row>
-    <row r="66" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>65</v>
       </c>
@@ -2083,7 +1876,7 @@
         <v>1061.0560696558241</v>
       </c>
     </row>
-    <row r="67" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>66</v>
       </c>
@@ -2097,7 +1890,7 @@
         <v>1061.0560696558241</v>
       </c>
     </row>
-    <row r="68" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>67</v>
       </c>
@@ -2111,7 +1904,7 @@
         <v>1765.8616993113646</v>
       </c>
     </row>
-    <row r="69" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>68</v>
       </c>
@@ -2125,7 +1918,7 @@
         <v>1765.8616993113646</v>
       </c>
     </row>
-    <row r="70" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>69</v>
       </c>
@@ -2139,7 +1932,7 @@
         <v>1765.8616993113646</v>
       </c>
     </row>
-    <row r="71" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>70</v>
       </c>
@@ -2153,7 +1946,7 @@
         <v>1765.8616993113646</v>
       </c>
     </row>
-    <row r="72" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>71</v>
       </c>
@@ -2167,7 +1960,7 @@
         <v>1765.8616993113646</v>
       </c>
     </row>
-    <row r="73" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A73">
         <v>72</v>
       </c>
@@ -2181,7 +1974,7 @@
         <v>1765.8616993113646</v>
       </c>
     </row>
-    <row r="74" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A74">
         <v>73</v>
       </c>
@@ -2195,7 +1988,7 @@
         <v>805.59139158107155</v>
       </c>
     </row>
-    <row r="75" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>74</v>
       </c>
@@ -2209,7 +2002,7 @@
         <v>805.59139158107155</v>
       </c>
     </row>
-    <row r="76" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>75</v>
       </c>
@@ -2223,7 +2016,7 @@
         <v>1346.5903878328372</v>
       </c>
     </row>
-    <row r="77" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>76</v>
       </c>
@@ -2237,7 +2030,7 @@
         <v>1346.5903878328372</v>
       </c>
     </row>
-    <row r="78" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>77</v>
       </c>
@@ -2251,7 +2044,7 @@
         <v>1346.5903878328372</v>
       </c>
     </row>
-    <row r="79" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>78</v>
       </c>
@@ -2265,7 +2058,7 @@
         <v>1346.5903878328372</v>
       </c>
     </row>
-    <row r="80" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>79</v>
       </c>
@@ -2279,7 +2072,7 @@
         <v>1346.5903878328372</v>
       </c>
     </row>
-    <row r="81" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>80</v>
       </c>
@@ -2293,7 +2086,7 @@
         <v>1346.5903878328372</v>
       </c>
     </row>
-    <row r="82" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>81</v>
       </c>
@@ -2307,7 +2100,7 @@
         <v>582.85678708808337</v>
       </c>
     </row>
-    <row r="83" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>82</v>
       </c>
@@ -2321,7 +2114,7 @@
         <v>582.85678708808337</v>
       </c>
     </row>
-    <row r="84" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>83</v>
       </c>
@@ -2335,7 +2128,7 @@
         <v>977.89718261795042</v>
       </c>
     </row>
-    <row r="85" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>84</v>
       </c>
@@ -2349,7 +2142,7 @@
         <v>977.89718261795042</v>
       </c>
     </row>
-    <row r="86" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>85</v>
       </c>
@@ -2363,7 +2156,7 @@
         <v>977.89718261795042</v>
       </c>
     </row>
-    <row r="87" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>86</v>
       </c>
@@ -2377,7 +2170,7 @@
         <v>977.89718261795042</v>
       </c>
     </row>
-    <row r="88" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>87</v>
       </c>
@@ -2391,7 +2184,7 @@
         <v>977.89718261795042</v>
       </c>
     </row>
-    <row r="89" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>88</v>
       </c>
@@ -2405,7 +2198,7 @@
         <v>977.89718261795042</v>
       </c>
     </row>
-    <row r="90" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>89</v>
       </c>
@@ -2419,7 +2212,7 @@
         <v>427.23885158421308</v>
       </c>
     </row>
-    <row r="91" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>90</v>
       </c>
@@ -2433,7 +2226,7 @@
         <v>427.23885158421308</v>
       </c>
     </row>
-    <row r="92" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>91</v>
       </c>
@@ -2447,7 +2240,7 @@
         <v>718.60297792286565</v>
       </c>
     </row>
-    <row r="93" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>92</v>
       </c>
@@ -2461,7 +2254,7 @@
         <v>718.60297792286565</v>
       </c>
     </row>
-    <row r="94" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>93</v>
       </c>
@@ -2475,7 +2268,7 @@
         <v>718.60297792286565</v>
       </c>
     </row>
-    <row r="95" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>94</v>
       </c>
@@ -2489,7 +2282,7 @@
         <v>718.60297792286565</v>
       </c>
     </row>
-    <row r="96" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>95</v>
       </c>
@@ -2503,7 +2296,7 @@
         <v>718.60297792286565</v>
       </c>
     </row>
-    <row r="97" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>96</v>
       </c>

</xml_diff>